<commit_message>
Add capacity tracking and LLM integration
</commit_message>
<xml_diff>
--- a/data/staffing_register.xlsx
+++ b/data/staffing_register.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Allocations" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Opportunities'!$A$1:$N$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Allocations'!$A$1:$I$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Opportunities'!$A$1:$N$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Allocations'!$A$1:$I$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1290,8 +1290,148 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>OPP-2026-012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Healthcare analytics delivery</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Axerion Pharma</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Build patient-level analytics and reporting for delivery teams.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2026-12-12</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>4</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Oncology</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Adherence | Patient Reach | Service Level</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Asia/Kolkata</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>No travel</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>OPP-2026-013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Healthcare analytics delivery</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Axerion Pharma</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Build patient-level analytics and reporting for delivery teams.</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2026-12-13</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>3</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Oncology</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Adherence | Patient Reach | Service Level</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Asia/Kolkata</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>No travel</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N12"/>
+  <autoFilter ref="A1:N14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1302,7 +1442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1922,8 +2062,137 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>EMP-1001</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Aarav Sharma</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>OPP-2026-012</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Healthcare analytics delivery</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>21.25</v>
+      </c>
+      <c r="F15" t="n">
+        <v>50</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2026-12-12</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>EMP-1238</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Kabir Khan</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>OPP-2026-013</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Healthcare analytics delivery</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>30</v>
+      </c>
+      <c r="F16" t="n">
+        <v>70.59999999999999</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2026-12-13</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>EMP-1172</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Neha Mehta</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>OPP-2026-013</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Healthcare analytics delivery</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>10</v>
+      </c>
+      <c r="F17" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-12-13</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I14"/>
+  <autoFilter ref="A1:I17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>